<commit_message>
Logiciel - Options de calcul pour les cas de charges
</commit_message>
<xml_diff>
--- a/TU/TU Section TestUnit_ProprietesSectionMixtePRS_MMoins.xlsx
+++ b/TU/TU Section TestUnit_ProprietesSectionMixtePRS_MMoins.xlsx
@@ -33,6 +33,7 @@
     <definedName name="Nw">Feuil1!$M$7</definedName>
     <definedName name="p">Feuil1!$K$15</definedName>
     <definedName name="PhiS">Feuil1!$E$19</definedName>
+    <definedName name="pLoc">Feuil1!$J$31</definedName>
     <definedName name="Td">Feuil1!$E$14</definedName>
     <definedName name="Tf">Feuil1!$E$6</definedName>
     <definedName name="Tw">Feuil1!$E$7</definedName>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="45">
   <si>
     <t>Profilé</t>
   </si>
@@ -103,6 +104,9 @@
     <t>Esp</t>
   </si>
   <si>
+    <t>z</t>
+  </si>
+  <si>
     <t>zGlobal</t>
   </si>
   <si>
@@ -179,13 +183,17 @@
   </si>
   <si>
     <t>MplRd</t>
+  </si>
+  <si>
+    <t>Résultante</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
@@ -266,7 +274,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -302,10 +310,17 @@
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="1" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -588,10 +603,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="C3:N32"/>
+  <dimension ref="C3:Q39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="3:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C3" s="1" t="s">
         <v>0</v>
       </c>
@@ -599,10 +614,10 @@
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="I3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="3:13" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D4" s="2" t="s">
         <v>1</v>
       </c>
@@ -613,19 +628,19 @@
         <v>6</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="3:13" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D5" s="2" t="s">
         <v>2</v>
       </c>
@@ -636,7 +651,7 @@
         <v>6</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K5" s="9" t="s">
         <v>6</v>
@@ -645,10 +660,10 @@
         <v>12</v>
       </c>
       <c r="M5" s="9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="3:13" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D6" s="2" t="s">
         <v>3</v>
       </c>
@@ -659,7 +674,7 @@
         <v>6</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J6" s="4">
         <f>Bf*Tf</f>
@@ -670,15 +685,18 @@
         <v>15</v>
       </c>
       <c r="L6" s="4">
-        <f>Fy/GammaM0</f>
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="M6" s="4">
         <f>J6*L6/1000</f>
-        <v>2475</v>
-      </c>
-    </row>
-    <row r="7" spans="3:13" x14ac:dyDescent="0.25">
+        <v>2385</v>
+      </c>
+      <c r="O6">
+        <f>-Ha+K6</f>
+        <v>-785</v>
+      </c>
+    </row>
+    <row r="7" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D7" s="2" t="s">
         <v>4</v>
       </c>
@@ -689,7 +707,7 @@
         <v>6</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J7" s="4">
         <f>Hw*Tw</f>
@@ -700,15 +718,22 @@
         <v>400</v>
       </c>
       <c r="L7" s="4">
-        <f>Fy/GammaM0</f>
         <v>275</v>
       </c>
       <c r="M7" s="10">
         <f t="shared" ref="M7:M10" si="0">J7*L7/1000</f>
         <v>3052.5</v>
       </c>
-    </row>
-    <row r="8" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="O7">
+        <f>-Ha+K7</f>
+        <v>-400</v>
+      </c>
+      <c r="Q7">
+        <f>J7/1000^2</f>
+        <v>1.11E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D8" s="2" t="s">
         <v>5</v>
       </c>
@@ -720,7 +745,7 @@
         <v>6</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J8" s="4">
         <f>Bf*Tf</f>
@@ -731,15 +756,19 @@
         <v>785</v>
       </c>
       <c r="L8" s="4">
-        <f>Fy/GammaM0</f>
-        <v>275</v>
+        <f>L6</f>
+        <v>265</v>
       </c>
       <c r="M8" s="4">
         <f t="shared" si="0"/>
-        <v>2475</v>
-      </c>
-    </row>
-    <row r="9" spans="3:13" x14ac:dyDescent="0.25">
+        <v>2385</v>
+      </c>
+      <c r="O8">
+        <f>-Ha+K8</f>
+        <v>-15</v>
+      </c>
+    </row>
+    <row r="9" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D9" s="2" t="s">
         <v>13</v>
       </c>
@@ -768,10 +797,14 @@
         <f t="shared" si="0"/>
         <v>8500</v>
       </c>
-    </row>
-    <row r="10" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="O9">
+        <f>-Ha+K9</f>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="10" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D10" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E10" s="5">
         <v>1</v>
@@ -795,8 +828,16 @@
         <f t="shared" si="0"/>
         <v>1365.9098493868667</v>
       </c>
-    </row>
-    <row r="12" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="O10">
+        <f>-Ha+K10</f>
+        <v>220</v>
+      </c>
+      <c r="Q10">
+        <f>J10/1000^2</f>
+        <v>3.1415926535897933E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C12" s="1" t="s">
         <v>7</v>
       </c>
@@ -807,17 +848,17 @@
         <v>0</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K12" s="4">
         <f>2*Nf+Nw</f>
-        <v>8002.5</v>
+        <v>7822.5</v>
       </c>
       <c r="L12" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="3:13" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D13" s="7" t="s">
         <v>8</v>
       </c>
@@ -828,7 +869,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="3:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D14" s="7" t="s">
         <v>9</v>
       </c>
@@ -839,7 +880,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="3:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D15" s="7" t="s">
         <v>11</v>
       </c>
@@ -850,36 +891,40 @@
         <v>12</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K15" s="12">
         <f>(Nw+Ns)/2/Nw</f>
         <v>0.72373625706582589</v>
       </c>
     </row>
-    <row r="16" spans="3:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="3:17" x14ac:dyDescent="0.25">
       <c r="D16" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E16" s="5">
         <v>1.5</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="K16" s="13">
+        <v>37</v>
+      </c>
+      <c r="K16" s="14">
         <f>p*Hw+Tf</f>
         <v>565.56483022871112</v>
       </c>
-    </row>
-    <row r="17" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="M16">
+        <f>Ha-zANP</f>
+        <v>234.43516977128888</v>
+      </c>
+    </row>
+    <row r="17" spans="3:15" x14ac:dyDescent="0.25">
       <c r="J17" s="8"/>
       <c r="K17" s="3"/>
     </row>
-    <row r="18" spans="3:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C18" s="1" t="s">
         <v>10</v>
       </c>
@@ -887,19 +932,19 @@
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="J18" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L18" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="M18" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="19" spans="3:14" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19" spans="3:15" x14ac:dyDescent="0.25">
       <c r="D19" s="7" t="s">
         <v>14</v>
       </c>
@@ -910,7 +955,7 @@
         <v>6</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K19" s="9" t="s">
         <v>6</v>
@@ -919,10 +964,10 @@
         <v>6</v>
       </c>
       <c r="M19" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="20" spans="3:14" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="20" spans="3:15" x14ac:dyDescent="0.25">
       <c r="D20" s="7" t="s">
         <v>15</v>
       </c>
@@ -933,11 +978,11 @@
         <v>6</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J20" s="10">
         <f>Nf</f>
-        <v>2475</v>
+        <v>2385</v>
       </c>
       <c r="K20" s="4">
         <f>Tf/2</f>
@@ -949,10 +994,14 @@
       </c>
       <c r="M20" s="10">
         <f>J20*L20/1000</f>
-        <v>1362.6479548160598</v>
-      </c>
-    </row>
-    <row r="21" spans="3:14" x14ac:dyDescent="0.25">
+        <v>1313.0971200954759</v>
+      </c>
+      <c r="O20" s="16">
+        <f>SUM(J20:J21)-SUM(J22:J24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="3:15" x14ac:dyDescent="0.25">
       <c r="D21" s="7" t="s">
         <v>16</v>
       </c>
@@ -963,7 +1012,7 @@
         <v>6</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="J21" s="10">
         <f>p*Nw</f>
@@ -982,9 +1031,9 @@
         <v>591.58623021693563</v>
       </c>
     </row>
-    <row r="22" spans="3:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:15" x14ac:dyDescent="0.25">
       <c r="D22" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E22" s="6">
         <f>Td-zArma</f>
@@ -994,7 +1043,7 @@
         <v>6</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J22" s="10">
         <f>(1-p)*Nw</f>
@@ -1013,20 +1062,20 @@
         <v>86.199585943794887</v>
       </c>
     </row>
-    <row r="23" spans="3:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:15" x14ac:dyDescent="0.25">
       <c r="D23" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E23" s="6">
         <f>Beff/EspBar</f>
         <v>10</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J23" s="10">
         <f>Nf</f>
-        <v>2475</v>
+        <v>2385</v>
       </c>
       <c r="K23" s="10">
         <f>Ha-Tf/2</f>
@@ -1038,12 +1087,12 @@
       </c>
       <c r="M23" s="10">
         <f t="shared" si="1"/>
-        <v>543.10204518393994</v>
-      </c>
-    </row>
-    <row r="24" spans="3:14" x14ac:dyDescent="0.25">
+        <v>523.352879904524</v>
+      </c>
+    </row>
+    <row r="24" spans="3:15" x14ac:dyDescent="0.25">
       <c r="D24" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E24" s="5">
         <v>500</v>
@@ -1071,57 +1120,136 @@
         <v>620.71747429839638</v>
       </c>
     </row>
-    <row r="25" spans="3:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:15" x14ac:dyDescent="0.25">
       <c r="D25" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E25" s="5">
         <v>1.1499999999999999</v>
       </c>
       <c r="J25" s="8"/>
-      <c r="K25" s="14"/>
-    </row>
-    <row r="26" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="K25" s="15"/>
+    </row>
+    <row r="26" spans="3:15" x14ac:dyDescent="0.25">
       <c r="E26" s="3"/>
       <c r="J26" s="8"/>
       <c r="K26" s="3"/>
       <c r="L26" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M26" s="10">
         <f>SUM(M20:M24)</f>
-        <v>3204.2532904591262</v>
+        <v>3134.9532904591269</v>
       </c>
       <c r="N26" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="27" spans="3:14" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="27" spans="3:15" x14ac:dyDescent="0.25">
       <c r="E27" s="3"/>
       <c r="J27" s="8"/>
       <c r="K27" s="3"/>
     </row>
-    <row r="28" spans="3:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:15" x14ac:dyDescent="0.25">
       <c r="E28" s="3"/>
       <c r="J28" s="8"/>
       <c r="K28" s="3"/>
     </row>
-    <row r="29" spans="3:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:15" x14ac:dyDescent="0.25">
       <c r="E29" s="3"/>
       <c r="J29" s="8"/>
       <c r="K29" s="3"/>
     </row>
-    <row r="30" spans="3:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:15" x14ac:dyDescent="0.25">
       <c r="E30" s="3"/>
-      <c r="K30" s="3"/>
-    </row>
-    <row r="31" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="I30" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="J30" s="5">
+        <f>-275</f>
+        <v>-275</v>
+      </c>
+      <c r="K30" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="3:15" x14ac:dyDescent="0.25">
       <c r="E31" s="3"/>
-      <c r="K31" s="3"/>
-    </row>
-    <row r="32" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="I31" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="J31" s="13">
+        <f>(Hw+J30+Tf)/Hw</f>
+        <v>0.66891891891891897</v>
+      </c>
+      <c r="K31" s="17">
+        <f>1-pLoc</f>
+        <v>0.33108108108108103</v>
+      </c>
+    </row>
+    <row r="32" spans="3:15" x14ac:dyDescent="0.25">
       <c r="E32" s="3"/>
       <c r="K32" s="3"/>
+    </row>
+    <row r="33" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="I33" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="J33" s="3">
+        <f>-Nf</f>
+        <v>-2385</v>
+      </c>
+    </row>
+    <row r="34" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="I34" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="J34" s="15">
+        <f>-pLoc*Nw</f>
+        <v>-2041.8750000000002</v>
+      </c>
+    </row>
+    <row r="35" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="I35" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="J35" s="15">
+        <f>(1-pLoc)*Nw</f>
+        <v>1010.6249999999999</v>
+      </c>
+    </row>
+    <row r="36" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="I36" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="J36" s="15">
+        <f>Nf</f>
+        <v>2385</v>
+      </c>
+    </row>
+    <row r="37" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="I37" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J37" s="15">
+        <f>+Ns</f>
+        <v>1365.9098493868667</v>
+      </c>
+    </row>
+    <row r="38" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="J38" s="16"/>
+    </row>
+    <row r="39" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="I39" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="J39" s="10">
+        <f>SUM(J33:J37)</f>
+        <v>334.65984938686665</v>
+      </c>
+      <c r="K39" t="s">
+        <v>32</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>